<commit_message>
docs: complete AI worklog and audit trail for SWR302 lab
</commit_message>
<xml_diff>
--- a/AI_AuditLog_Example.xlsx
+++ b/AI_AuditLog_Example.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23016" windowHeight="9048"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23016" windowHeight="9048" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="1. Metadata &amp; Summary" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="209">
   <si>
     <t>AI AUDIT LOG - METADATA &amp; SUMMARY</t>
   </si>
@@ -451,6 +451,213 @@
   </si>
   <si>
     <t>Car Maintenance &amp; Service Booking System</t>
+  </si>
+  <si>
+    <t>Decision Support</t>
+  </si>
+  <si>
+    <t>Assignment 1a - MoSCoW Prioritization</t>
+  </si>
+  <si>
+    <t>Needed to prioritize 10 requirements for a clinic appointment booking MVP with only 3 developers and an 8-week deadline.</t>
+  </si>
+  <si>
+    <t>How should I classify the clinic booking requirements using the MoSCoW method?</t>
+  </si>
+  <si>
+    <t>AI suggested prioritizing booking-related functions as Must Have and postponing reporting and advanced features.</t>
+  </si>
+  <si>
+    <t>I used the AI response as an initial reference only. I reviewed each requirement based on business value, project scope, and implementation effort. I learned that MoSCoW classification must be aligned with MVP objectives rather than feature popularity.</t>
+  </si>
+  <si>
+    <t>Final MoSCoW classification table in Assignment 1a.</t>
+  </si>
+  <si>
+    <t>Requirement Analysis</t>
+  </si>
+  <si>
+    <t>Assignment 1a - R02</t>
+  </si>
+  <si>
+    <t>Uncertainty whether doctor schedule viewing on mobile should be Won't Have or Should Have.</t>
+  </si>
+  <si>
+    <t>Should doctor schedule viewing on mobile be classified as Won't Have or Should Have in an MVP?</t>
+  </si>
+  <si>
+    <t>AI recommended Should Have because doctors still need access to appointment schedules.</t>
+  </si>
+  <si>
+    <t>Initially, I considered Won't Have because of the limited development resources. After reviewing the clinic workflow, I realized doctors still require appointment visibility. I accepted the AI recommendation but refined it by stating that web access can temporarily replace a dedicated mobile application.</t>
+  </si>
+  <si>
+    <t>Assignment 1a - R07</t>
+  </si>
+  <si>
+    <t>Needed to determine the priority of online payment integration.</t>
+  </si>
+  <si>
+    <t>Is online payment a Must Have feature for a clinic booking MVP?</t>
+  </si>
+  <si>
+    <t>AI suggested Could Have because patients can still pay at the clinic.</t>
+  </si>
+  <si>
+    <t>I did not accept the suggestion immediately. I compared the business importance of booking appointments versus payment processing. Since appointment booking remains possible without online payment, I agreed with the AI recommendation and classified it as Could Have.</t>
+  </si>
+  <si>
+    <t>Requirement Validation</t>
+  </si>
+  <si>
+    <t>Assignment 1b - Games People Play</t>
+  </si>
+  <si>
+    <t>Needed BA-style questions to challenge requirement assumptions.</t>
+  </si>
+  <si>
+    <t>Generate Games People Play questions for SMS appointment reminders.</t>
+  </si>
+  <si>
+    <t>AI proposed questions related to reminder timing and alternative communication methods.</t>
+  </si>
+  <si>
+    <t>I reviewed the generated questions and modified them to better fit the clinic environment. I focused on identifying workarounds and understanding whether SMS reminders provide essential business value.</t>
+  </si>
+  <si>
+    <t>Scope Reduction</t>
+  </si>
+  <si>
+    <t>Assignment 1c - Deadline Reduction</t>
+  </si>
+  <si>
+    <t>Needed to identify which requirements should be downgraded when the project duration is reduced from 8 weeks to 5 weeks.</t>
+  </si>
+  <si>
+    <t>Which requirements should be downgraded if the deadline is shortened to 5 weeks?</t>
+  </si>
+  <si>
+    <t>AI suggested removing SMS reminders and management reporting from the MVP scope.</t>
+  </si>
+  <si>
+    <t>I evaluated whether each feature had a manual workaround. Since receptionists can manually remind patients and managers can temporarily use raw data exports, I accepted the recommendation. This reinforced the importance of protecting core business functionality during scope reduction.</t>
+  </si>
+  <si>
+    <t>Concept Learning</t>
+  </si>
+  <si>
+    <t>Assignment 2a - Verification vs Validation</t>
+  </si>
+  <si>
+    <t>Needed a clear understanding of Verification and Validation before analyzing the scenarios.</t>
+  </si>
+  <si>
+    <t>Explain the difference between Verification and Validation with software examples.</t>
+  </si>
+  <si>
+    <t>AI explained that Verification means building the product right, while Validation means building the right product.</t>
+  </si>
+  <si>
+    <t>I used the explanation to strengthen my understanding of the concepts. Instead of copying the answer directly, I applied the definitions independently to each scenario. This helped me connect theory with practical examples.</t>
+  </si>
+  <si>
+    <t>Root Cause Analysis</t>
+  </si>
+  <si>
+    <t>Assignment 2b - TH5</t>
+  </si>
+  <si>
+    <t>Needed to explain why all automated tests passed but the customer still rejected the system.</t>
+  </si>
+  <si>
+    <t>Why can a software project pass all tests but still fail customer acceptance?</t>
+  </si>
+  <si>
+    <t>AI explained that Verification may succeed while Validation fails if requirements do not reflect actual business needs.</t>
+  </si>
+  <si>
+    <t>I extended the AI explanation using the clinic example involving mandatory CMND and BHYT fields. I realized that successful testing cannot compensate for poorly validated requirements. This helped me better understand the role of Validation activities before implementation.</t>
+  </si>
+  <si>
+    <t>Final classification of R02 as Should Have.</t>
+  </si>
+  <si>
+    <t>Final classification of R07 as Could Have.</t>
+  </si>
+  <si>
+    <t>Final questions for R03.</t>
+  </si>
+  <si>
+    <t>Assignment 1c final prioritization changes.</t>
+  </si>
+  <si>
+    <t>Assignment 2a classification table.</t>
+  </si>
+  <si>
+    <t>TH5 detailed analysis section.</t>
+  </si>
+  <si>
+    <t>Acceptance Criteria Generation</t>
+  </si>
+  <si>
+    <t>Assignment 3a</t>
+  </si>
+  <si>
+    <t>Needed to write Given-When-Then acceptance criteria for online appointment booking.</t>
+  </si>
+  <si>
+    <t>Generate acceptance criteria for a patient appointment booking user story.</t>
+  </si>
+  <si>
+    <t>AI generated several acceptance criteria covering successful booking and validation scenarios.</t>
+  </si>
+  <si>
+    <t>I reviewed all generated criteria and removed those that were not directly related to the user story. I refined the final acceptance criteria to ensure they were testable, measurable, and aligned with the business objective.</t>
+  </si>
+  <si>
+    <t>Final Acceptance Criteria 1–4.</t>
+  </si>
+  <si>
+    <t>Risk Identification</t>
+  </si>
+  <si>
+    <t>Assignment 3b</t>
+  </si>
+  <si>
+    <t>Needed an example of an acceptance criterion that is commonly overlooked.</t>
+  </si>
+  <si>
+    <t>What acceptance criteria are often forgotten in appointment booking systems?</t>
+  </si>
+  <si>
+    <t>AI identified concurrency and overbooking scenarios.</t>
+  </si>
+  <si>
+    <t>I analyzed the recommendation and concluded that concurrency is a realistic operational risk. I selected this example because it demonstrates deeper requirement analysis and highlights system behavior under real-world conditions.</t>
+  </si>
+  <si>
+    <t>Assignment 3b discussion.</t>
+  </si>
+  <si>
+    <t>Test Design</t>
+  </si>
+  <si>
+    <t>Assignment 3c</t>
+  </si>
+  <si>
+    <t>Needed to create a detailed test case for a fully booked appointment timeslot.</t>
+  </si>
+  <si>
+    <t>Generate a test case for a fully booked appointment slot.</t>
+  </si>
+  <si>
+    <t>AI provided preconditions, steps, test data, and expected results.</t>
+  </si>
+  <si>
+    <t>I improved the generated test case by adding more detailed test data, clarifying expected outcomes, and ensuring traceability to the acceptance criterion. This made the test case more practical and realistic.</t>
+  </si>
+  <si>
+    <t>TC_BOOK_002 test case.</t>
   </si>
 </sst>
 </file>
@@ -590,7 +797,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -642,6 +849,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1179,11 +1389,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="3" width="18" customWidth="1"/>
+    <col min="2" max="2" width="30.77734375" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
     <col min="4" max="4" width="25" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
     <col min="6" max="6" width="35" customWidth="1"/>
@@ -1242,8 +1453,8 @@
       </c>
     </row>
     <row r="4" spans="1:8" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="7" t="s">
-        <v>49</v>
+      <c r="A4" s="7">
+        <v>1</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>50</v>
@@ -1268,8 +1479,8 @@
       </c>
     </row>
     <row r="5" spans="1:8" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="7" t="s">
-        <v>56</v>
+      <c r="A5" s="7">
+        <v>2</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>57</v>
@@ -1294,8 +1505,8 @@
       </c>
     </row>
     <row r="6" spans="1:8" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="7" t="s">
-        <v>63</v>
+      <c r="A6" s="7">
+        <v>3</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>64</v>
@@ -1320,104 +1531,264 @@
       </c>
     </row>
     <row r="7" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="7"/>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
+      <c r="A7" s="24">
+        <v>4</v>
+      </c>
+      <c r="B7" s="24" t="s">
+        <v>140</v>
+      </c>
+      <c r="C7" s="24" t="s">
+        <v>141</v>
+      </c>
+      <c r="D7" s="24" t="s">
+        <v>142</v>
+      </c>
+      <c r="E7" s="24" t="s">
+        <v>143</v>
+      </c>
+      <c r="F7" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="G7" s="24" t="s">
+        <v>145</v>
+      </c>
+      <c r="H7" s="24" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="8" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="7"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
+      <c r="A8" s="24">
+        <v>5</v>
+      </c>
+      <c r="B8" s="24" t="s">
+        <v>147</v>
+      </c>
+      <c r="C8" s="24" t="s">
+        <v>148</v>
+      </c>
+      <c r="D8" s="24" t="s">
+        <v>149</v>
+      </c>
+      <c r="E8" s="24" t="s">
+        <v>150</v>
+      </c>
+      <c r="F8" s="24" t="s">
+        <v>151</v>
+      </c>
+      <c r="G8" s="24" t="s">
+        <v>152</v>
+      </c>
+      <c r="H8" s="24" t="s">
+        <v>182</v>
+      </c>
     </row>
     <row r="9" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="7"/>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
+      <c r="A9" s="24">
+        <v>6</v>
+      </c>
+      <c r="B9" s="24" t="s">
+        <v>147</v>
+      </c>
+      <c r="C9" s="24" t="s">
+        <v>153</v>
+      </c>
+      <c r="D9" s="24" t="s">
+        <v>154</v>
+      </c>
+      <c r="E9" s="24" t="s">
+        <v>155</v>
+      </c>
+      <c r="F9" s="24" t="s">
+        <v>156</v>
+      </c>
+      <c r="G9" s="24" t="s">
+        <v>157</v>
+      </c>
+      <c r="H9" s="24" t="s">
+        <v>183</v>
+      </c>
     </row>
     <row r="10" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
+      <c r="A10" s="24">
+        <v>7</v>
+      </c>
+      <c r="B10" s="24" t="s">
+        <v>158</v>
+      </c>
+      <c r="C10" s="24" t="s">
+        <v>159</v>
+      </c>
+      <c r="D10" s="24" t="s">
+        <v>160</v>
+      </c>
+      <c r="E10" s="24" t="s">
+        <v>161</v>
+      </c>
+      <c r="F10" s="24" t="s">
+        <v>162</v>
+      </c>
+      <c r="G10" s="24" t="s">
+        <v>163</v>
+      </c>
+      <c r="H10" s="24" t="s">
+        <v>184</v>
+      </c>
     </row>
     <row r="11" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="7"/>
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
-      <c r="H11" s="7"/>
+      <c r="A11" s="24">
+        <v>8</v>
+      </c>
+      <c r="B11" s="24" t="s">
+        <v>164</v>
+      </c>
+      <c r="C11" s="24" t="s">
+        <v>165</v>
+      </c>
+      <c r="D11" s="24" t="s">
+        <v>166</v>
+      </c>
+      <c r="E11" s="24" t="s">
+        <v>167</v>
+      </c>
+      <c r="F11" s="24" t="s">
+        <v>168</v>
+      </c>
+      <c r="G11" s="24" t="s">
+        <v>169</v>
+      </c>
+      <c r="H11" s="24" t="s">
+        <v>185</v>
+      </c>
     </row>
     <row r="12" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="7"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7"/>
+      <c r="A12" s="24">
+        <v>9</v>
+      </c>
+      <c r="B12" s="24" t="s">
+        <v>170</v>
+      </c>
+      <c r="C12" s="24" t="s">
+        <v>171</v>
+      </c>
+      <c r="D12" s="24" t="s">
+        <v>172</v>
+      </c>
+      <c r="E12" s="24" t="s">
+        <v>173</v>
+      </c>
+      <c r="F12" s="24" t="s">
+        <v>174</v>
+      </c>
+      <c r="G12" s="24" t="s">
+        <v>175</v>
+      </c>
+      <c r="H12" s="24" t="s">
+        <v>186</v>
+      </c>
     </row>
     <row r="13" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="7"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
+      <c r="A13" s="24">
+        <v>10</v>
+      </c>
+      <c r="B13" s="24" t="s">
+        <v>176</v>
+      </c>
+      <c r="C13" s="24" t="s">
+        <v>177</v>
+      </c>
+      <c r="D13" s="24" t="s">
+        <v>178</v>
+      </c>
+      <c r="E13" s="24" t="s">
+        <v>179</v>
+      </c>
+      <c r="F13" s="24" t="s">
+        <v>180</v>
+      </c>
+      <c r="G13" s="24" t="s">
+        <v>181</v>
+      </c>
+      <c r="H13" s="24" t="s">
+        <v>187</v>
+      </c>
     </row>
     <row r="14" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="7"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
-      <c r="H14" s="7"/>
+      <c r="A14" s="24">
+        <v>11</v>
+      </c>
+      <c r="B14" s="24" t="s">
+        <v>188</v>
+      </c>
+      <c r="C14" s="24" t="s">
+        <v>189</v>
+      </c>
+      <c r="D14" s="24" t="s">
+        <v>190</v>
+      </c>
+      <c r="E14" s="24" t="s">
+        <v>191</v>
+      </c>
+      <c r="F14" s="24" t="s">
+        <v>192</v>
+      </c>
+      <c r="G14" s="24" t="s">
+        <v>193</v>
+      </c>
+      <c r="H14" s="24" t="s">
+        <v>194</v>
+      </c>
     </row>
     <row r="15" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="7"/>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7"/>
-      <c r="H15" s="7"/>
+      <c r="A15" s="24">
+        <v>12</v>
+      </c>
+      <c r="B15" s="24" t="s">
+        <v>195</v>
+      </c>
+      <c r="C15" s="24" t="s">
+        <v>196</v>
+      </c>
+      <c r="D15" s="24" t="s">
+        <v>197</v>
+      </c>
+      <c r="E15" s="24" t="s">
+        <v>198</v>
+      </c>
+      <c r="F15" s="24" t="s">
+        <v>199</v>
+      </c>
+      <c r="G15" s="24" t="s">
+        <v>200</v>
+      </c>
+      <c r="H15" s="24" t="s">
+        <v>201</v>
+      </c>
     </row>
     <row r="16" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="7"/>
-      <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
-      <c r="H16" s="7"/>
+      <c r="A16" s="24">
+        <v>13</v>
+      </c>
+      <c r="B16" s="24" t="s">
+        <v>202</v>
+      </c>
+      <c r="C16" s="24" t="s">
+        <v>203</v>
+      </c>
+      <c r="D16" s="24" t="s">
+        <v>204</v>
+      </c>
+      <c r="E16" s="24" t="s">
+        <v>205</v>
+      </c>
+      <c r="F16" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="G16" s="24" t="s">
+        <v>207</v>
+      </c>
+      <c r="H16" s="24" t="s">
+        <v>208</v>
+      </c>
     </row>
     <row r="17" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7"/>
@@ -1508,16 +1879,6 @@
       <c r="F25" s="7"/>
       <c r="G25" s="7"/>
       <c r="H25" s="7"/>
-    </row>
-    <row r="26" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="7"/>
-      <c r="B26" s="7"/>
-      <c r="C26" s="7"/>
-      <c r="D26" s="7"/>
-      <c r="E26" s="7"/>
-      <c r="F26" s="7"/>
-      <c r="G26" s="7"/>
-      <c r="H26" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>